<commit_message>
add group member 2 information
</commit_message>
<xml_diff>
--- a/STA380GroupForm.xlsx
+++ b/STA380GroupForm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chr1sren/Documents/CodeCourse/sta380_repo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jasmi\Desktop\Study\2025-2026\Winter\sta380_repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BB423E-DEBE-CB41-BB4B-94C5247AED6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C140A3-4321-491B-A505-69C46209DD43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -88,9 +88,6 @@
     <t>To report an inactive member, please refer to the "Reporting Inactive Members" section under the project description.</t>
   </si>
   <si>
-    <t>Team Cheryl</t>
-  </si>
-  <si>
     <t>Renfei Wu</t>
   </si>
   <si>
@@ -110,6 +107,21 @@
   </si>
   <si>
     <t>Robustness of models with different loss functions and estators under distribution shift</t>
+  </si>
+  <si>
+    <t>Team Chris</t>
+  </si>
+  <si>
+    <t>Shiqi Tian</t>
+  </si>
+  <si>
+    <t>tianshi8</t>
+  </si>
+  <si>
+    <t>https://github.com/Dream-ABC</t>
+  </si>
+  <si>
+    <t>Dream-ABC</t>
   </si>
 </sst>
 </file>
@@ -187,7 +199,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -404,17 +416,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" customWidth="1"/>
-    <col min="4" max="4" width="18.1640625" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" customWidth="1"/>
     <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.1640625" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -422,15 +434,15 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -438,76 +450,76 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
     </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="3" t="s">
         <v>8</v>
@@ -525,62 +537,77 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="D21">
         <v>1009998237</v>
       </c>
       <c r="E21" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21" t="s">
         <v>25</v>
       </c>
-      <c r="F21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22">
+        <v>1009834654</v>
+      </c>
+      <c r="E22" t="s">
+        <v>33</v>
+      </c>
+      <c r="F22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>21</v>
       </c>

</xml_diff>